<commit_message>
updating json files with new data from gas packs data.xlsx
</commit_message>
<xml_diff>
--- a/DATA/DATA FILES/GAS PACKS DATA.xlsx
+++ b/DATA/DATA FILES/GAS PACKS DATA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex.schwindt\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hoffmanandhoffman-my.sharepoint.com/personal/alex_schwindt_hoffman-hoffman_com/Documents/Desktop/Quick Select App Version 3/DATA/DATA FILES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD341DD-89F0-4EFC-955D-A302FBB6E9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2FD341DD-89F0-4EFC-955D-A302FBB6E9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DAD0148-2A00-4060-B5D4-F91DC7E89F32}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SCHEDULE" sheetId="1" r:id="rId1"/>
@@ -790,7 +790,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -799,29 +799,29 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1161,7 +1161,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" style="1" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.42578125" style="1" customWidth="1"/>
     <col min="4" max="4" width="6.85546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="10.28515625" style="1" customWidth="1"/>
@@ -1206,7 +1206,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:51" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="22" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="23"/>
@@ -1233,7 +1233,7 @@
       <c r="W1" s="23"/>
       <c r="X1" s="23"/>
       <c r="Y1" s="24"/>
-      <c r="AA1" s="29" t="s">
+      <c r="AA1" s="28" t="s">
         <v>8</v>
       </c>
       <c r="AB1" s="23"/>
@@ -1242,7 +1242,7 @@
       <c r="AE1" s="23"/>
       <c r="AF1" s="24"/>
       <c r="AG1" s="16"/>
-      <c r="AH1" s="28" t="s">
+      <c r="AH1" s="22" t="s">
         <v>9</v>
       </c>
       <c r="AI1" s="23"/>
@@ -1264,7 +1264,7 @@
       <c r="AY1" s="24"/>
     </row>
     <row r="2" spans="1:51" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="35" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="23"/>
@@ -1291,22 +1291,22 @@
       <c r="W2" s="23"/>
       <c r="X2" s="23"/>
       <c r="Y2" s="24"/>
-      <c r="AA2" s="29" t="s">
+      <c r="AA2" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="AB2" s="29" t="s">
+      <c r="AB2" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="AC2" s="29" t="s">
+      <c r="AC2" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="AD2" s="29" t="s">
+      <c r="AD2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="AE2" s="29" t="s">
+      <c r="AE2" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="AF2" s="29" t="s">
+      <c r="AF2" s="28" t="s">
         <v>16</v>
       </c>
       <c r="AG2" s="16"/>
@@ -1366,49 +1366,49 @@
       </c>
     </row>
     <row r="3" spans="1:51" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="32"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="31" t="s">
+      <c r="E3" s="30"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="31" t="s">
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="33"/>
-      <c r="S3" s="36" t="s">
+      <c r="O3" s="30"/>
+      <c r="P3" s="30"/>
+      <c r="Q3" s="30"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="T3" s="34" t="s">
+      <c r="T3" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="U3" s="31" t="s">
+      <c r="U3" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="V3" s="32"/>
-      <c r="W3" s="32"/>
-      <c r="X3" s="33"/>
-      <c r="Y3" s="34" t="s">
+      <c r="V3" s="30"/>
+      <c r="W3" s="30"/>
+      <c r="X3" s="31"/>
+      <c r="Y3" s="27" t="s">
         <v>43</v>
       </c>
       <c r="AA3" s="26"/>
@@ -1501,12 +1501,12 @@
         <v>62</v>
       </c>
       <c r="Y4" s="26"/>
-      <c r="AA4" s="30"/>
-      <c r="AB4" s="30"/>
-      <c r="AC4" s="30"/>
-      <c r="AD4" s="30"/>
-      <c r="AE4" s="30"/>
-      <c r="AF4" s="30"/>
+      <c r="AA4" s="33"/>
+      <c r="AB4" s="33"/>
+      <c r="AC4" s="33"/>
+      <c r="AD4" s="33"/>
+      <c r="AE4" s="33"/>
+      <c r="AF4" s="33"/>
       <c r="AG4" s="16"/>
       <c r="AH4" s="26"/>
       <c r="AI4" s="26"/>
@@ -7525,6 +7525,28 @@
     <row r="126" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="AY2:AY4"/>
+    <mergeCell ref="AN2:AN4"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="AA2:AA4"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="AC2:AC4"/>
+    <mergeCell ref="AW2:AW4"/>
+    <mergeCell ref="AX2:AX4"/>
+    <mergeCell ref="A2:Y2"/>
+    <mergeCell ref="AS2:AS4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="AT2:AT4"/>
+    <mergeCell ref="AK2:AK4"/>
+    <mergeCell ref="AM2:AM4"/>
+    <mergeCell ref="AO2:AO4"/>
+    <mergeCell ref="AU2:AU4"/>
+    <mergeCell ref="AP2:AP4"/>
+    <mergeCell ref="AF2:AF4"/>
+    <mergeCell ref="AR2:AR4"/>
+    <mergeCell ref="AH2:AH4"/>
+    <mergeCell ref="AI2:AI4"/>
     <mergeCell ref="A1:Y1"/>
     <mergeCell ref="AJ2:AJ4"/>
     <mergeCell ref="T3:T4"/>
@@ -7541,28 +7563,6 @@
     <mergeCell ref="AB2:AB4"/>
     <mergeCell ref="AD2:AD4"/>
     <mergeCell ref="AH1:AY1"/>
-    <mergeCell ref="AP2:AP4"/>
-    <mergeCell ref="AF2:AF4"/>
-    <mergeCell ref="AR2:AR4"/>
-    <mergeCell ref="AH2:AH4"/>
-    <mergeCell ref="AI2:AI4"/>
-    <mergeCell ref="AT2:AT4"/>
-    <mergeCell ref="AK2:AK4"/>
-    <mergeCell ref="AM2:AM4"/>
-    <mergeCell ref="AO2:AO4"/>
-    <mergeCell ref="AU2:AU4"/>
-    <mergeCell ref="AW2:AW4"/>
-    <mergeCell ref="AX2:AX4"/>
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="AS2:AS4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="AY2:AY4"/>
-    <mergeCell ref="AN2:AN4"/>
-    <mergeCell ref="N3:R3"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="AA2:AA4"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="AC2:AC4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>